<commit_message>
commiting screenshot and report files
</commit_message>
<xml_diff>
--- a/src/main/resources/testdata.xlsx
+++ b/src/main/resources/testdata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\eclipse-workspace\AmazonJavaLearnings\Demoblaze\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF995B3D-E4A3-445F-B5BF-67295401DCB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0237A9F4-ED48-41AF-9200-DA5A4F128391}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21060" windowHeight="18495" activeTab="4" xr2:uid="{FB42E33F-6F13-442B-AAF2-108A22EDAF15}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21060" windowHeight="18495" activeTab="3" xr2:uid="{FB42E33F-6F13-442B-AAF2-108A22EDAF15}"/>
   </bookViews>
   <sheets>
     <sheet name="Registration" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="70">
   <si>
     <t>Username</t>
   </si>
@@ -128,6 +128,126 @@
   </si>
   <si>
     <t>ASUS Full HD</t>
+  </si>
+  <si>
+    <t>ProductName</t>
+  </si>
+  <si>
+    <t>Action</t>
+  </si>
+  <si>
+    <t>Samsung galaxy s6</t>
+  </si>
+  <si>
+    <t>Nokia lumia 1520</t>
+  </si>
+  <si>
+    <t>Add</t>
+  </si>
+  <si>
+    <t>Remove</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add </t>
+  </si>
+  <si>
+    <t>User Type</t>
+  </si>
+  <si>
+    <t>Shipping Address</t>
+  </si>
+  <si>
+    <t>Payment Method</t>
+  </si>
+  <si>
+    <t>Expected Message</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>City</t>
+  </si>
+  <si>
+    <t>Month</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>Registered</t>
+  </si>
+  <si>
+    <t>Guest</t>
+  </si>
+  <si>
+    <t>123 Main St, NY</t>
+  </si>
+  <si>
+    <t>456 Elm St, CA</t>
+  </si>
+  <si>
+    <t>789 Oadk St, TX</t>
+  </si>
+  <si>
+    <t>321 Pine St, FL</t>
+  </si>
+  <si>
+    <t>Credit Card</t>
+  </si>
+  <si>
+    <t>PayPal</t>
+  </si>
+  <si>
+    <t>Debit Card</t>
+  </si>
+  <si>
+    <t>Thank you for your purchase!</t>
+  </si>
+  <si>
+    <t>Shipping address required</t>
+  </si>
+  <si>
+    <t>Payment method required</t>
+  </si>
+  <si>
+    <t>GuestUser1</t>
+  </si>
+  <si>
+    <t>RegisteredUser1</t>
+  </si>
+  <si>
+    <t>GuestUser2</t>
+  </si>
+  <si>
+    <t>GuestUser3</t>
+  </si>
+  <si>
+    <t>RegisteredUser2</t>
+  </si>
+  <si>
+    <t>US</t>
+  </si>
+  <si>
+    <t>NY</t>
+  </si>
+  <si>
+    <t>CA</t>
+  </si>
+  <si>
+    <t>TX</t>
+  </si>
+  <si>
+    <t>FL</t>
+  </si>
+  <si>
+    <t>Expected Total Price</t>
+  </si>
+  <si>
+    <t>Expected Item Count</t>
   </si>
 </sst>
 </file>
@@ -186,16 +306,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -522,30 +638,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="3" t="b">
+      <c r="D2" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -565,136 +681,136 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="3" t="b">
+      <c r="D2" s="2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="3" t="b">
+      <c r="D3" s="2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="3" t="b">
+      <c r="D4" s="2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="3" t="b">
+      <c r="D5" s="2" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="3" t="b">
+      <c r="D6" s="2" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="3" t="b">
+      <c r="D7" s="2" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3" t="s">
+      <c r="B8" s="2"/>
+      <c r="C8" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="3" t="b">
+      <c r="D8" s="2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3" t="s">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D9" s="3" t="b">
+      <c r="D9" s="2" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="3" t="b">
+      <c r="D10" s="2" t="b">
         <v>1</v>
       </c>
     </row>
@@ -713,58 +829,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="2" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="2" t="s">
         <v>23</v>
       </c>
     </row>
@@ -775,18 +891,289 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A651EC7D-DF39-4068-8DD5-BA9497C764AB}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" s="2">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" s="2">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0</v>
+      </c>
+      <c r="D4" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="2">
+        <v>1</v>
+      </c>
+      <c r="D5" s="2">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" s="2">
+        <v>0</v>
+      </c>
+      <c r="D6" s="2">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D387EBFA-35B4-4351-93E3-24EB2E056B9C}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="H2" s="2">
+        <v>10</v>
+      </c>
+      <c r="I2" s="2">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="H3" s="2">
+        <v>10</v>
+      </c>
+      <c r="I3" s="2">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2">
+        <v>10</v>
+      </c>
+      <c r="I4" s="2">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="H5" s="2">
+        <v>10</v>
+      </c>
+      <c r="I5" s="2">
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="H6" s="2">
+        <v>10</v>
+      </c>
+      <c r="I6" s="2">
+        <v>2025</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>